<commit_message>
Updated with final video and updated with final agenda
</commit_message>
<xml_diff>
--- a/config/Agenda.xlsx
+++ b/config/Agenda.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Travel Guide - Avolta Customer\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Travel Guide - Avolta Customer\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7530" firstSheet="2" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930" firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Client Profile" sheetId="1" state="hidden" r:id="rId1"/>
     <sheet name="Objective" sheetId="6" state="hidden" r:id="rId2"/>
     <sheet name="Objective_Visit" sheetId="10" r:id="rId3"/>
     <sheet name="Office Visit Plan_Updated" sheetId="9" r:id="rId4"/>
-    <sheet name="Config" sheetId="12" r:id="rId5"/>
+    <sheet name="Config" sheetId="11" r:id="rId5"/>
     <sheet name="Logistics" sheetId="4" state="hidden" r:id="rId6"/>
     <sheet name="Office Visit Plan - Old" sheetId="3" state="hidden" r:id="rId7"/>
   </sheets>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="175">
   <si>
     <t>Client Name</t>
   </si>
@@ -326,25 +326,12 @@
     <t>Changepond Corporate Overiew</t>
   </si>
   <si>
-    <t>Changepond Leadership Update</t>
-  </si>
-  <si>
     <t>Manuel &amp; Ino</t>
   </si>
   <si>
     <t>Changepond Participants</t>
   </si>
   <si>
-    <t>New Initiatives - Demo</t>
-  </si>
-  <si>
-    <t>POC 1 : Dynamic Personalized Offer Engine
-POC 2 : Shop by Emotion
-POC 3 :Real time operational Dashboard view 
-POC 4 : Orders screen - Intelligent priority sorting using color coding 
-POC 5 : QA POC's</t>
-  </si>
-  <si>
     <t>Ideathon 2.0</t>
   </si>
   <si>
@@ -358,9 +345,6 @@
   </si>
   <si>
     <t>Avolta's roadmap, priorities, expectations and understand potential areas for collaboration</t>
-  </si>
-  <si>
-    <t>Balaji D, Nagaraj / Sara</t>
   </si>
   <si>
     <t>Prize Distribution</t>
@@ -404,18 +388,6 @@
     <t xml:space="preserve">Team Building at Turf </t>
   </si>
   <si>
-    <t>Balaji D, Nagaraj</t>
-  </si>
-  <si>
-    <t>Akhilesh, Gopal, Sakthivel</t>
-  </si>
-  <si>
-    <t>Team</t>
-  </si>
-  <si>
-    <t>Leadership Team</t>
-  </si>
-  <si>
     <t>Changepond's experience in offering QA Organizatin setup for other customer - Our Approach, Framework &amp; Methodology, AI in QA Offerings, Governance &amp; Metrics, Risk &amp; Challenges</t>
   </si>
   <si>
@@ -440,9 +412,6 @@
     <t>Discussion: Use of AI for knowledge acquisition in OMS—AI can extract functional flows, identify dependencies, map integrations, and summarize key features. This discussion aims to clarify what is expected, who will benefit, and how these outcomes can be achieved.</t>
   </si>
   <si>
-    <t xml:space="preserve">Topic 5 : CLAP Framework - Agentic Model </t>
-  </si>
-  <si>
     <t>Live demo on how CLAP can build an application from a prototype to a fully functional application</t>
   </si>
   <si>
@@ -452,9 +421,6 @@
     <t>Interaction with the team : What went well in 2026 and what are the improvements</t>
   </si>
   <si>
-    <t>OMS Team</t>
-  </si>
-  <si>
     <t>Godwin &amp; Prasath</t>
   </si>
   <si>
@@ -470,9 +436,6 @@
     <t>Finalize the Best Ideas from the Brainstorming Session with Avolta</t>
   </si>
   <si>
-    <t>Topic 5: To be decided</t>
-  </si>
-  <si>
     <t>Next Steps</t>
   </si>
   <si>
@@ -480,9 +443,6 @@
   </si>
   <si>
     <t>Dinner with Changepond Leadership Team</t>
-  </si>
-  <si>
-    <t>Topic 4 : Accelerate Knowledge Acquisition Techniques (Use of AI)</t>
   </si>
   <si>
     <t>Topic</t>
@@ -515,6 +475,112 @@
   </si>
   <si>
     <t>Coffee Break, Tree Planting. Facility Visit (GCC), Team Photo</t>
+  </si>
+  <si>
+    <t>Changepond Leadership Presentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Topic 4 : CLAP Framework - Agentic Model </t>
+  </si>
+  <si>
+    <t>Topic 5 : Accelerate Knowledge Acquisition Techniques (Use of AI)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Akhilesh, Gopal, </t>
+  </si>
+  <si>
+    <t>Gopal</t>
+  </si>
+  <si>
+    <t>Krishna Prasath</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kishore </t>
+  </si>
+  <si>
+    <t>New Initiatives - Demo &amp; Predictive Intelligience Dashboard</t>
+  </si>
+  <si>
+    <t>Pothy /KalaRaj</t>
+  </si>
+  <si>
+    <t>Topic 6: (Placeholder - Topic TBD)</t>
+  </si>
+  <si>
+    <t>Balaji D, Nagaraj , Sara, Katta</t>
+  </si>
+  <si>
+    <t>Anil, Selva, SaravanaPandy , Sara</t>
+  </si>
+  <si>
+    <t>Akhilesh, Gopal, Sara, Selva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selva or Dhinkar or SP </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sara ,
+( Have to check the Availability of Leadership team) </t>
+  </si>
+  <si>
+    <t>Sara, Selva, Danny, Godwin , KrishnaPrasath , Dhinakar, Amol</t>
+  </si>
+  <si>
+    <t>Sara, Selva,  Godwin , KrishnaPrasath , Prasath</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kalaraj , Pothy, Sara, Selva </t>
+  </si>
+  <si>
+    <t>Amol</t>
+  </si>
+  <si>
+    <t>OMS team , Sara, Selva</t>
+  </si>
+  <si>
+    <t>Sara, Selva, SP,</t>
+  </si>
+  <si>
+    <t>David /Amol</t>
+  </si>
+  <si>
+    <t>Sara, Selva, Amol, Akhilesh ,Dhinakar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prize disttibution to Team 
+Memento to Clients </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entire Team </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Predictive Intelligience Dashboard
+POC 1 : Dynamic Personalized Offer Engine
+POC 2 : Shop by Emotion
+POC 3 :Real time operational Dashboard view 
+POC 4 : Orders screen - Intelligent priority sorting using color coding 
+</t>
+  </si>
+  <si>
+    <t>Selva, SP, Dhinakar</t>
+  </si>
+  <si>
+    <t>Session Presenter</t>
+  </si>
+  <si>
+    <t>Session Owner</t>
+  </si>
+  <si>
+    <t>Kishore</t>
+  </si>
+  <si>
+    <t>Catering Facility</t>
+  </si>
+  <si>
+    <t>Catering Facility , Admin</t>
+  </si>
+  <si>
+    <t>Balaji D, Nagaraj ,  Katta, Anil</t>
   </si>
   <si>
     <t xml:space="preserve">Sheet name </t>
@@ -615,13 +681,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor rgb="FFD9E1F2"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -653,7 +719,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -725,9 +791,54 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="21" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="21" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -741,45 +852,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1169,13 +1241,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.45">
       <c r="A1" s="22" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="80" x14ac:dyDescent="0.45">
@@ -1183,10 +1255,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="80" x14ac:dyDescent="0.35">
@@ -1194,10 +1266,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="64" x14ac:dyDescent="0.45">
@@ -1205,10 +1277,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="48" x14ac:dyDescent="0.45">
@@ -1216,10 +1288,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -1230,1005 +1302,1144 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.26953125" style="28" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.54296875" style="32" customWidth="1"/>
-    <col min="3" max="3" width="11.26953125" style="30" customWidth="1"/>
+    <col min="1" max="1" width="24.54296875" style="43" customWidth="1"/>
+    <col min="2" max="2" width="10" style="47" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" style="45" customWidth="1"/>
     <col min="4" max="4" width="11.1796875" style="20" customWidth="1"/>
     <col min="5" max="5" width="42.1796875" style="21" customWidth="1"/>
     <col min="6" max="6" width="56.7265625" style="21" customWidth="1"/>
-    <col min="7" max="7" width="20.7265625" style="21" customWidth="1"/>
-    <col min="8" max="8" width="17.453125" style="21" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="17.453125" style="21" customWidth="1"/>
-    <col min="11" max="11" width="25.54296875" style="21" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="21" style="21" hidden="1" customWidth="1"/>
-    <col min="13" max="14" width="7" style="21" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="10.453125" style="21" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="54.453125" style="21" hidden="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.1796875" style="21"/>
+    <col min="7" max="8" width="20.7265625" style="21" customWidth="1"/>
+    <col min="9" max="9" width="17.453125" style="21" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="17.453125" style="21" customWidth="1"/>
+    <col min="12" max="12" width="25.54296875" style="21" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="21" style="21" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="7" style="21" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="10.453125" style="21" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="54.453125" style="21" hidden="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.1796875" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="20" customFormat="1" ht="49.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+    <row r="1" spans="1:17" s="20" customFormat="1" ht="49.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="34" t="s">
-        <v>148</v>
-      </c>
-      <c r="C1" s="33" t="s">
+      <c r="B1" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="35" t="s">
+      <c r="F1" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="35" t="s">
+      <c r="G1" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="H1" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="I1" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="35" t="s">
-        <v>94</v>
-      </c>
-      <c r="J1" s="35" t="s">
+      <c r="J1" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="K1" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="K1" s="36" t="s">
+      <c r="L1" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="36" t="s">
+      <c r="M1" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="36" t="s">
+      <c r="N1" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="36" t="s">
+      <c r="O1" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="36" t="s">
+      <c r="P1" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="P1" s="36" t="s">
+      <c r="Q1" s="30" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="27" customFormat="1" ht="33" x14ac:dyDescent="0.35">
-      <c r="A2" s="37">
+    <row r="2" spans="1:17" s="36" customFormat="1" ht="33" x14ac:dyDescent="0.35">
+      <c r="A2" s="31">
         <v>46083</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="39">
+      <c r="B2" s="32"/>
+      <c r="C2" s="33">
         <v>0.14583333333333334</v>
       </c>
-      <c r="D2" s="39">
+      <c r="D2" s="33">
         <v>0.1875</v>
       </c>
-      <c r="E2" s="40" t="s">
+      <c r="E2" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="F2" s="40" t="s">
-        <v>104</v>
-      </c>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-    </row>
-    <row r="3" spans="1:16" s="27" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="37">
+      <c r="F2" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+    </row>
+    <row r="3" spans="1:17" s="36" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="31">
         <v>46083</v>
       </c>
-      <c r="B3" s="42">
+      <c r="B3" s="37">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="C3" s="39">
+      <c r="C3" s="33">
         <v>0.4375</v>
       </c>
-      <c r="D3" s="39">
+      <c r="D3" s="33">
         <f>C3+B3</f>
         <v>0.45833333333333331</v>
       </c>
-      <c r="E3" s="40" t="s">
+      <c r="E3" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="41"/>
-      <c r="L3" s="41"/>
-      <c r="M3" s="41"/>
-      <c r="N3" s="41"/>
-      <c r="O3" s="41"/>
-      <c r="P3" s="41"/>
-    </row>
-    <row r="4" spans="1:16" ht="49.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="37">
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34" t="s">
+        <v>41</v>
+      </c>
+      <c r="I3" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="34" t="s">
+        <v>41</v>
+      </c>
+      <c r="K3" s="34"/>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
+      <c r="N3" s="35"/>
+      <c r="O3" s="35"/>
+      <c r="P3" s="35"/>
+      <c r="Q3" s="35"/>
+    </row>
+    <row r="4" spans="1:17" ht="49.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="31">
         <v>46083</v>
       </c>
-      <c r="B4" s="42">
+      <c r="B4" s="37">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="C4" s="39">
+      <c r="C4" s="33">
         <f>D3</f>
         <v>0.45833333333333331</v>
       </c>
-      <c r="D4" s="39">
+      <c r="D4" s="33">
         <f t="shared" ref="D4:D27" si="0">C4+B4</f>
         <v>0.47916666666666663</v>
       </c>
-      <c r="E4" s="43" t="s">
+      <c r="E4" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="43" t="s">
-        <v>106</v>
-      </c>
-      <c r="G4" s="43" t="s">
+      <c r="F4" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="H4" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="43"/>
-      <c r="J4" s="43"/>
-      <c r="K4" s="44" t="s">
+      <c r="G4" s="38"/>
+      <c r="H4" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="38" t="s">
+        <v>164</v>
+      </c>
+      <c r="K4" s="38"/>
+      <c r="L4" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="L4" s="44" t="s">
+      <c r="M4" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="M4" s="44" t="s">
+      <c r="N4" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="N4" s="44"/>
-      <c r="O4" s="44"/>
-      <c r="P4" s="44"/>
-    </row>
-    <row r="5" spans="1:16" ht="33" x14ac:dyDescent="0.35">
-      <c r="A5" s="37">
+      <c r="O4" s="39"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="39"/>
+    </row>
+    <row r="5" spans="1:17" ht="33" x14ac:dyDescent="0.35">
+      <c r="A5" s="31">
         <v>46083</v>
       </c>
-      <c r="B5" s="42">
+      <c r="B5" s="37">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="C5" s="39">
+      <c r="C5" s="33">
         <f t="shared" ref="C5:C10" si="1">D4</f>
         <v>0.47916666666666663</v>
       </c>
-      <c r="D5" s="39">
+      <c r="D5" s="33">
         <f t="shared" si="0"/>
         <v>0.49999999999999994</v>
       </c>
-      <c r="E5" s="43" t="s">
-        <v>100</v>
-      </c>
-      <c r="F5" s="45" t="s">
-        <v>101</v>
-      </c>
-      <c r="G5" s="43" t="s">
-        <v>93</v>
-      </c>
-      <c r="H5" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" s="43"/>
-      <c r="J5" s="43"/>
-      <c r="K5" s="44" t="s">
+      <c r="E5" s="38" t="s">
+        <v>97</v>
+      </c>
+      <c r="F5" s="40" t="s">
+        <v>98</v>
+      </c>
+      <c r="G5" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="H5" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="I5" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="K5" s="38"/>
+      <c r="L5" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="L5" s="44"/>
-      <c r="M5" s="44" t="s">
+      <c r="M5" s="39"/>
+      <c r="N5" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="N5" s="44"/>
-      <c r="O5" s="44"/>
-      <c r="P5" s="44"/>
-    </row>
-    <row r="6" spans="1:16" ht="33" x14ac:dyDescent="0.35">
-      <c r="A6" s="37">
+      <c r="O5" s="39"/>
+      <c r="P5" s="39"/>
+      <c r="Q5" s="39"/>
+    </row>
+    <row r="6" spans="1:17" ht="33" x14ac:dyDescent="0.35">
+      <c r="A6" s="31">
         <v>46083</v>
       </c>
-      <c r="B6" s="42">
+      <c r="B6" s="37">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="C6" s="39">
+      <c r="C6" s="33">
         <f t="shared" si="1"/>
         <v>0.49999999999999994</v>
       </c>
-      <c r="D6" s="39">
+      <c r="D6" s="33">
         <f t="shared" si="0"/>
         <v>0.52083333333333326</v>
       </c>
-      <c r="E6" s="43" t="s">
-        <v>92</v>
-      </c>
-      <c r="F6" s="45" t="s">
+      <c r="E6" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="F6" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="G6" s="43" t="s">
-        <v>116</v>
-      </c>
-      <c r="H6" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I6" s="43"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="44" t="s">
+      <c r="G6" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="38" t="s">
+        <v>170</v>
+      </c>
+      <c r="K6" s="38"/>
+      <c r="L6" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="L6" s="44"/>
-      <c r="M6" s="44" t="s">
+      <c r="M6" s="39"/>
+      <c r="N6" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="N6" s="44"/>
-      <c r="O6" s="44"/>
-      <c r="P6" s="44"/>
-    </row>
-    <row r="7" spans="1:16" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="37">
+      <c r="O6" s="39"/>
+      <c r="P6" s="39"/>
+      <c r="Q6" s="39"/>
+    </row>
+    <row r="7" spans="1:17" ht="33" x14ac:dyDescent="0.35">
+      <c r="A7" s="31">
         <v>46083</v>
       </c>
-      <c r="B7" s="42">
+      <c r="B7" s="37">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="C7" s="39">
+      <c r="C7" s="33">
         <f t="shared" si="1"/>
         <v>0.52083333333333326</v>
       </c>
-      <c r="D7" s="39">
+      <c r="D7" s="33">
         <f t="shared" si="0"/>
         <v>0.56249999999999989</v>
       </c>
-      <c r="E7" s="43" t="s">
+      <c r="E7" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="43" t="s">
-        <v>105</v>
-      </c>
-      <c r="G7" s="43" t="s">
-        <v>116</v>
-      </c>
-      <c r="H7" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="43"/>
-      <c r="J7" s="43"/>
-      <c r="K7" s="44"/>
-      <c r="L7" s="44"/>
-      <c r="M7" s="44"/>
-      <c r="N7" s="44"/>
-      <c r="O7" s="44"/>
-      <c r="P7" s="44"/>
-    </row>
-    <row r="8" spans="1:16" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="37">
+      <c r="F7" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="G7" s="38" t="s">
+        <v>168</v>
+      </c>
+      <c r="H7" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="I7" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="38" t="s">
+        <v>148</v>
+      </c>
+      <c r="K7" s="38"/>
+      <c r="L7" s="39"/>
+      <c r="M7" s="39"/>
+      <c r="N7" s="39"/>
+      <c r="O7" s="39"/>
+      <c r="P7" s="39"/>
+      <c r="Q7" s="39"/>
+    </row>
+    <row r="8" spans="1:17" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="31">
         <v>46083</v>
       </c>
-      <c r="B8" s="42">
+      <c r="B8" s="37">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="C8" s="39">
+      <c r="C8" s="33">
         <f t="shared" si="1"/>
         <v>0.56249999999999989</v>
       </c>
-      <c r="D8" s="39">
+      <c r="D8" s="33">
         <f t="shared" si="0"/>
         <v>0.60416666666666652</v>
       </c>
-      <c r="E8" s="43" t="s">
-        <v>136</v>
-      </c>
-      <c r="F8" s="45" t="s">
-        <v>120</v>
-      </c>
-      <c r="G8" s="43" t="s">
-        <v>134</v>
-      </c>
-      <c r="H8" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I8" s="43"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="44"/>
-      <c r="L8" s="44"/>
-      <c r="M8" s="44"/>
-      <c r="N8" s="44"/>
-      <c r="O8" s="44"/>
-      <c r="P8" s="44"/>
-    </row>
-    <row r="9" spans="1:16" ht="82.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="37">
+      <c r="E8" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="F8" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="G8" s="38" t="s">
+        <v>124</v>
+      </c>
+      <c r="H8" s="38" t="s">
+        <v>74</v>
+      </c>
+      <c r="I8" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="K8" s="38"/>
+      <c r="L8" s="39"/>
+      <c r="M8" s="39"/>
+      <c r="N8" s="39"/>
+      <c r="O8" s="39"/>
+      <c r="P8" s="39"/>
+      <c r="Q8" s="39"/>
+    </row>
+    <row r="9" spans="1:17" ht="82.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="31">
         <v>46083</v>
       </c>
-      <c r="B9" s="42">
+      <c r="B9" s="37">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="C9" s="39">
+      <c r="C9" s="33">
         <f t="shared" si="1"/>
         <v>0.60416666666666652</v>
       </c>
-      <c r="D9" s="39">
+      <c r="D9" s="33">
         <f t="shared" si="0"/>
         <v>0.62499999999999989</v>
       </c>
-      <c r="E9" s="43" t="s">
-        <v>121</v>
-      </c>
-      <c r="F9" s="43" t="s">
-        <v>122</v>
-      </c>
-      <c r="G9" s="43" t="s">
-        <v>117</v>
-      </c>
-      <c r="H9" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I9" s="43"/>
-      <c r="J9" s="43"/>
-      <c r="K9" s="44"/>
-      <c r="L9" s="44"/>
-      <c r="M9" s="44"/>
-      <c r="N9" s="44"/>
-      <c r="O9" s="44"/>
-      <c r="P9" s="44"/>
-    </row>
-    <row r="10" spans="1:16" ht="66" x14ac:dyDescent="0.35">
-      <c r="A10" s="37">
+      <c r="E9" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="F9" s="38" t="s">
+        <v>114</v>
+      </c>
+      <c r="G9" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="H9" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="I9" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J9" s="38" t="s">
+        <v>150</v>
+      </c>
+      <c r="K9" s="38"/>
+      <c r="L9" s="39"/>
+      <c r="M9" s="39"/>
+      <c r="N9" s="39"/>
+      <c r="O9" s="39"/>
+      <c r="P9" s="39"/>
+      <c r="Q9" s="39"/>
+    </row>
+    <row r="10" spans="1:17" ht="66" x14ac:dyDescent="0.35">
+      <c r="A10" s="31">
         <v>46083</v>
       </c>
-      <c r="B10" s="42">
+      <c r="B10" s="37">
         <v>6.25E-2</v>
       </c>
-      <c r="C10" s="39">
+      <c r="C10" s="33">
         <f t="shared" si="1"/>
         <v>0.62499999999999989</v>
       </c>
-      <c r="D10" s="39">
+      <c r="D10" s="33">
         <f t="shared" si="0"/>
         <v>0.68749999999999989</v>
       </c>
-      <c r="E10" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="F10" s="45" t="s">
-        <v>124</v>
-      </c>
-      <c r="G10" s="43"/>
-      <c r="H10" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I10" s="43"/>
-      <c r="J10" s="43"/>
-      <c r="K10" s="44"/>
-      <c r="L10" s="44"/>
-      <c r="M10" s="44"/>
-      <c r="N10" s="44"/>
-      <c r="O10" s="44"/>
-      <c r="P10" s="44"/>
-    </row>
-    <row r="11" spans="1:16" ht="82.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="37">
+      <c r="E10" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="F10" s="40" t="s">
+        <v>116</v>
+      </c>
+      <c r="G10" s="38"/>
+      <c r="H10" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="I10" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J10" s="38" t="s">
+        <v>151</v>
+      </c>
+      <c r="K10" s="38"/>
+      <c r="L10" s="39"/>
+      <c r="M10" s="39"/>
+      <c r="N10" s="39"/>
+      <c r="O10" s="39"/>
+      <c r="P10" s="39"/>
+      <c r="Q10" s="39"/>
+    </row>
+    <row r="11" spans="1:17" ht="82.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="31">
         <v>46083</v>
       </c>
-      <c r="B11" s="42">
+      <c r="B11" s="37">
         <v>0.10416666666666667</v>
       </c>
-      <c r="C11" s="39">
+      <c r="C11" s="33">
         <f>D10</f>
         <v>0.68749999999999989</v>
       </c>
-      <c r="D11" s="39">
+      <c r="D11" s="33">
         <f t="shared" si="0"/>
         <v>0.79166666666666652</v>
       </c>
-      <c r="E11" s="43" t="s">
+      <c r="E11" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="45" t="s">
-        <v>125</v>
-      </c>
-      <c r="G11" s="43"/>
-      <c r="H11" s="43"/>
-      <c r="I11" s="43"/>
-      <c r="J11" s="43"/>
-      <c r="K11" s="44"/>
-      <c r="L11" s="44"/>
-      <c r="M11" s="44"/>
-      <c r="N11" s="44"/>
-      <c r="O11" s="44"/>
-      <c r="P11" s="44"/>
-    </row>
-    <row r="12" spans="1:16" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="37">
+      <c r="F11" s="40" t="s">
+        <v>117</v>
+      </c>
+      <c r="G11" s="38"/>
+      <c r="H11" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="I11" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J11" s="38" t="s">
+        <v>151</v>
+      </c>
+      <c r="K11" s="38"/>
+      <c r="L11" s="39"/>
+      <c r="M11" s="39"/>
+      <c r="N11" s="39"/>
+      <c r="O11" s="39"/>
+      <c r="P11" s="39"/>
+      <c r="Q11" s="39"/>
+    </row>
+    <row r="12" spans="1:17" ht="66" x14ac:dyDescent="0.35">
+      <c r="A12" s="31">
         <v>46083</v>
       </c>
-      <c r="B12" s="42">
+      <c r="B12" s="37">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="C12" s="39">
+      <c r="C12" s="33">
         <f>D11</f>
         <v>0.79166666666666652</v>
       </c>
-      <c r="D12" s="39">
+      <c r="D12" s="33">
         <f t="shared" si="0"/>
         <v>0.83333333333333315</v>
       </c>
-      <c r="E12" s="43" t="s">
-        <v>141</v>
-      </c>
-      <c r="F12" s="43" t="s">
-        <v>140</v>
-      </c>
-      <c r="G12" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="H12" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
-      <c r="K12" s="44"/>
-      <c r="L12" s="44"/>
-      <c r="M12" s="44"/>
-      <c r="N12" s="44"/>
-      <c r="O12" s="44"/>
-      <c r="P12" s="44"/>
-    </row>
-    <row r="13" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="37">
+      <c r="E12" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="F12" s="38" t="s">
+        <v>129</v>
+      </c>
+      <c r="G12" s="38"/>
+      <c r="H12" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="I12" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J12" s="38" t="s">
+        <v>152</v>
+      </c>
+      <c r="K12" s="38"/>
+      <c r="L12" s="39"/>
+      <c r="M12" s="39"/>
+      <c r="N12" s="39"/>
+      <c r="O12" s="39"/>
+      <c r="P12" s="39"/>
+      <c r="Q12" s="39"/>
+    </row>
+    <row r="13" spans="1:17" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="42">
         <v>46084</v>
       </c>
-      <c r="B13" s="42">
+      <c r="B13" s="37">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="C13" s="39">
+      <c r="C13" s="33">
         <v>0.39583333333333331</v>
       </c>
-      <c r="D13" s="39">
+      <c r="D13" s="33">
         <f t="shared" si="0"/>
         <v>0.41666666666666663</v>
       </c>
-      <c r="E13" s="40" t="s">
+      <c r="E13" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="45"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I13" s="43"/>
-      <c r="J13" s="43"/>
-      <c r="K13" s="44"/>
-      <c r="L13" s="44"/>
-      <c r="M13" s="44"/>
-      <c r="N13" s="44"/>
-      <c r="O13" s="44"/>
-      <c r="P13" s="44"/>
-    </row>
-    <row r="14" spans="1:16" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="37">
+      <c r="F13" s="40"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="I13" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J13" s="38"/>
+      <c r="K13" s="38"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="39"/>
+      <c r="N13" s="39"/>
+      <c r="O13" s="39"/>
+      <c r="P13" s="39"/>
+      <c r="Q13" s="39"/>
+    </row>
+    <row r="14" spans="1:17" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="42">
         <v>46084</v>
       </c>
-      <c r="B14" s="42">
+      <c r="B14" s="37">
         <v>3.125E-2</v>
       </c>
-      <c r="C14" s="39">
+      <c r="C14" s="33">
         <f>D13</f>
         <v>0.41666666666666663</v>
       </c>
-      <c r="D14" s="39">
+      <c r="D14" s="33">
         <f t="shared" si="0"/>
         <v>0.44791666666666663</v>
       </c>
-      <c r="E14" s="43" t="s">
-        <v>107</v>
-      </c>
-      <c r="F14" s="43" t="s">
-        <v>126</v>
-      </c>
-      <c r="G14" s="43" t="s">
-        <v>99</v>
-      </c>
-      <c r="H14" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43"/>
-      <c r="K14" s="44"/>
-      <c r="L14" s="44"/>
-      <c r="M14" s="44"/>
-      <c r="N14" s="44"/>
-      <c r="O14" s="44"/>
-      <c r="P14" s="44"/>
-    </row>
-    <row r="15" spans="1:16" ht="33" x14ac:dyDescent="0.35">
-      <c r="A15" s="37">
+      <c r="E14" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="F14" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="G14" s="38" t="s">
+        <v>96</v>
+      </c>
+      <c r="H14" s="38" t="s">
+        <v>96</v>
+      </c>
+      <c r="I14" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J14" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="K14" s="38"/>
+      <c r="L14" s="39"/>
+      <c r="M14" s="39"/>
+      <c r="N14" s="39"/>
+      <c r="O14" s="39"/>
+      <c r="P14" s="39"/>
+      <c r="Q14" s="39"/>
+    </row>
+    <row r="15" spans="1:17" ht="66" x14ac:dyDescent="0.35">
+      <c r="A15" s="42">
         <v>46084</v>
       </c>
-      <c r="B15" s="42">
+      <c r="B15" s="37">
         <v>3.125E-2</v>
       </c>
-      <c r="C15" s="39">
+      <c r="C15" s="33">
         <f t="shared" ref="C15:C27" si="2">D14</f>
         <v>0.44791666666666663</v>
       </c>
-      <c r="D15" s="39">
+      <c r="D15" s="33">
         <f t="shared" si="0"/>
         <v>0.47916666666666663</v>
       </c>
-      <c r="E15" s="43" t="s">
-        <v>128</v>
-      </c>
-      <c r="F15" s="43" t="s">
-        <v>129</v>
-      </c>
-      <c r="G15" s="43" t="s">
-        <v>133</v>
-      </c>
-      <c r="H15" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="44"/>
-      <c r="L15" s="44"/>
-      <c r="M15" s="44"/>
-      <c r="N15" s="44"/>
-      <c r="O15" s="44"/>
-      <c r="P15" s="44"/>
-    </row>
-    <row r="16" spans="1:16" ht="33" x14ac:dyDescent="0.35">
-      <c r="A16" s="37">
+      <c r="E15" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="F15" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="G15" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="H15" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="I15" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J15" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="K15" s="38"/>
+      <c r="L15" s="39"/>
+      <c r="M15" s="39"/>
+      <c r="N15" s="39"/>
+      <c r="O15" s="39"/>
+      <c r="P15" s="39"/>
+      <c r="Q15" s="39"/>
+    </row>
+    <row r="16" spans="1:17" ht="33" x14ac:dyDescent="0.35">
+      <c r="A16" s="42">
         <v>46084</v>
       </c>
-      <c r="B16" s="42">
+      <c r="B16" s="37">
         <v>3.125E-2</v>
       </c>
-      <c r="C16" s="39">
+      <c r="C16" s="33">
         <f t="shared" si="2"/>
         <v>0.47916666666666663</v>
       </c>
-      <c r="D16" s="39">
+      <c r="D16" s="33">
         <f t="shared" si="0"/>
         <v>0.51041666666666663</v>
       </c>
-      <c r="E16" s="43" t="s">
-        <v>149</v>
-      </c>
-      <c r="F16" s="43"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="43"/>
-      <c r="I16" s="43"/>
-      <c r="J16" s="43"/>
-      <c r="K16" s="44"/>
-      <c r="L16" s="44"/>
-      <c r="M16" s="44"/>
-      <c r="N16" s="44"/>
-      <c r="O16" s="44"/>
-      <c r="P16" s="44"/>
-    </row>
-    <row r="17" spans="1:16" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="37">
+      <c r="E16" s="38" t="s">
+        <v>137</v>
+      </c>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="H16" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="I16" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J16" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="K16" s="38"/>
+      <c r="L16" s="39"/>
+      <c r="M16" s="39"/>
+      <c r="N16" s="39"/>
+      <c r="O16" s="39"/>
+      <c r="P16" s="39"/>
+      <c r="Q16" s="39"/>
+    </row>
+    <row r="17" spans="1:17" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="42">
         <v>46084</v>
       </c>
-      <c r="B17" s="42">
+      <c r="B17" s="37">
         <v>3.125E-2</v>
       </c>
-      <c r="C17" s="39">
+      <c r="C17" s="33">
         <f t="shared" si="2"/>
         <v>0.51041666666666663</v>
       </c>
-      <c r="D17" s="39">
+      <c r="D17" s="33">
         <f t="shared" si="0"/>
         <v>0.54166666666666663</v>
       </c>
-      <c r="E17" s="43" t="s">
-        <v>142</v>
-      </c>
-      <c r="F17" s="43" t="s">
-        <v>127</v>
-      </c>
-      <c r="G17" s="43" t="s">
-        <v>98</v>
-      </c>
-      <c r="H17" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I17" s="43"/>
-      <c r="J17" s="43"/>
-      <c r="K17" s="44"/>
-      <c r="L17" s="44"/>
-      <c r="M17" s="44"/>
-      <c r="N17" s="44"/>
-      <c r="O17" s="44"/>
-      <c r="P17" s="44"/>
-    </row>
-    <row r="18" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="37">
+      <c r="E17" s="38" t="s">
+        <v>140</v>
+      </c>
+      <c r="F17" s="38" t="s">
+        <v>119</v>
+      </c>
+      <c r="G17" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="H17" s="38" t="s">
+        <v>146</v>
+      </c>
+      <c r="I17" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J17" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="K17" s="38"/>
+      <c r="L17" s="39"/>
+      <c r="M17" s="39"/>
+      <c r="N17" s="39"/>
+      <c r="O17" s="39"/>
+      <c r="P17" s="39"/>
+      <c r="Q17" s="39"/>
+    </row>
+    <row r="18" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="42">
         <v>46084</v>
       </c>
-      <c r="B18" s="42">
+      <c r="B18" s="37">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="C18" s="39">
+      <c r="C18" s="33">
         <f t="shared" ref="C18:C26" si="3">D17</f>
         <v>0.54166666666666663</v>
       </c>
-      <c r="D18" s="39">
+      <c r="D18" s="33">
         <f t="shared" si="0"/>
         <v>0.58333333333333326</v>
       </c>
-      <c r="E18" s="43" t="s">
+      <c r="E18" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F18" s="43" t="s">
-        <v>105</v>
-      </c>
-      <c r="G18" s="43"/>
-      <c r="H18" s="43"/>
-      <c r="I18" s="43"/>
-      <c r="J18" s="43"/>
-      <c r="K18" s="44"/>
-      <c r="L18" s="44"/>
-      <c r="M18" s="44"/>
-      <c r="N18" s="44"/>
-      <c r="O18" s="44"/>
-      <c r="P18" s="44"/>
-    </row>
-    <row r="19" spans="1:16" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="37">
+      <c r="F18" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="G18" s="38" t="s">
+        <v>168</v>
+      </c>
+      <c r="H18" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="I18" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J18" s="38"/>
+      <c r="K18" s="38"/>
+      <c r="L18" s="39"/>
+      <c r="M18" s="39"/>
+      <c r="N18" s="39"/>
+      <c r="O18" s="39"/>
+      <c r="P18" s="39"/>
+      <c r="Q18" s="39"/>
+    </row>
+    <row r="19" spans="1:17" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="42">
         <v>46084</v>
       </c>
-      <c r="B19" s="42">
-        <v>3.125E-2</v>
-      </c>
-      <c r="C19" s="39">
+      <c r="B19" s="37">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="C19" s="33">
         <f t="shared" si="3"/>
         <v>0.58333333333333326</v>
       </c>
-      <c r="D19" s="39">
+      <c r="D19" s="33">
         <f>C19+B19</f>
-        <v>0.61458333333333326</v>
-      </c>
-      <c r="E19" s="43" t="s">
-        <v>138</v>
-      </c>
-      <c r="F19" s="45"/>
-      <c r="G19" s="43"/>
-      <c r="H19" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I19" s="43"/>
-      <c r="J19" s="43"/>
-      <c r="K19" s="44"/>
-      <c r="L19" s="44"/>
-      <c r="M19" s="44"/>
-      <c r="N19" s="44"/>
-      <c r="O19" s="44"/>
-      <c r="P19" s="44"/>
-    </row>
-    <row r="20" spans="1:16" ht="33" x14ac:dyDescent="0.35">
-      <c r="A20" s="37">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>147</v>
+      </c>
+      <c r="F19" s="40"/>
+      <c r="G19" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="H19" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="I19" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J19" s="38"/>
+      <c r="K19" s="38"/>
+      <c r="L19" s="39"/>
+      <c r="M19" s="39"/>
+      <c r="N19" s="39"/>
+      <c r="O19" s="39"/>
+      <c r="P19" s="39"/>
+      <c r="Q19" s="39"/>
+    </row>
+    <row r="20" spans="1:17" ht="33" x14ac:dyDescent="0.35">
+      <c r="A20" s="42">
         <v>46084</v>
       </c>
-      <c r="B20" s="42">
+      <c r="B20" s="37">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="C20" s="33">
+        <f t="shared" si="3"/>
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D20" s="33">
+        <f t="shared" si="0"/>
+        <v>0.625</v>
+      </c>
+      <c r="E20" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="F20" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="G20" s="38" t="s">
+        <v>156</v>
+      </c>
+      <c r="H20" s="38" t="s">
+        <v>72</v>
+      </c>
+      <c r="I20" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J20" s="38" t="s">
+        <v>157</v>
+      </c>
+      <c r="K20" s="38"/>
+      <c r="L20" s="39"/>
+      <c r="M20" s="39"/>
+      <c r="N20" s="39"/>
+      <c r="O20" s="39"/>
+      <c r="P20" s="39"/>
+      <c r="Q20" s="39"/>
+    </row>
+    <row r="21" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="42">
+        <v>46084</v>
+      </c>
+      <c r="B21" s="37">
+        <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="C21" s="33">
+        <f t="shared" si="3"/>
+        <v>0.625</v>
+      </c>
+      <c r="D21" s="33">
+        <f t="shared" ref="D21" si="4">C21+B21</f>
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="E21" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="F21" s="38"/>
+      <c r="G21" s="38" t="s">
+        <v>168</v>
+      </c>
+      <c r="H21" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="I21" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J21" s="38"/>
+      <c r="K21" s="38"/>
+      <c r="L21" s="39"/>
+      <c r="M21" s="39"/>
+      <c r="N21" s="39"/>
+      <c r="O21" s="39"/>
+      <c r="P21" s="39"/>
+      <c r="Q21" s="39"/>
+    </row>
+    <row r="22" spans="1:17" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="42">
+        <v>46084</v>
+      </c>
+      <c r="B22" s="37">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="C22" s="33">
+        <f t="shared" si="3"/>
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="D22" s="33">
+        <f t="shared" ref="D22" si="5">C22+B22</f>
+        <v>0.65625</v>
+      </c>
+      <c r="E22" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="F22" s="40"/>
+      <c r="G22" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="H22" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="I22" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J22" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="K22" s="38"/>
+      <c r="L22" s="39"/>
+      <c r="M22" s="39"/>
+      <c r="N22" s="39"/>
+      <c r="O22" s="39"/>
+      <c r="P22" s="39"/>
+      <c r="Q22" s="39"/>
+    </row>
+    <row r="23" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="42">
+        <v>46084</v>
+      </c>
+      <c r="B23" s="37">
         <v>3.125E-2</v>
       </c>
-      <c r="C20" s="39">
+      <c r="C23" s="33">
         <f t="shared" si="3"/>
-        <v>0.61458333333333326</v>
-      </c>
-      <c r="D20" s="39">
+        <v>0.65625</v>
+      </c>
+      <c r="D23" s="33">
         <f t="shared" si="0"/>
-        <v>0.64583333333333326</v>
-      </c>
-      <c r="E20" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="F20" s="45" t="s">
-        <v>131</v>
-      </c>
-      <c r="G20" s="43" t="s">
-        <v>132</v>
-      </c>
-      <c r="H20" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I20" s="43"/>
-      <c r="J20" s="43"/>
-      <c r="K20" s="44"/>
-      <c r="L20" s="44"/>
-      <c r="M20" s="44"/>
-      <c r="N20" s="44"/>
-      <c r="O20" s="44"/>
-      <c r="P20" s="44"/>
-    </row>
-    <row r="21" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="37">
+        <v>0.6875</v>
+      </c>
+      <c r="E23" s="38" t="s">
+        <v>145</v>
+      </c>
+      <c r="F23" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="G23" s="38" t="s">
+        <v>159</v>
+      </c>
+      <c r="H23" s="38" t="s">
+        <v>72</v>
+      </c>
+      <c r="I23" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J23" s="38" t="s">
+        <v>157</v>
+      </c>
+      <c r="K23" s="38"/>
+      <c r="L23" s="39"/>
+      <c r="M23" s="39"/>
+      <c r="N23" s="39"/>
+      <c r="O23" s="39"/>
+      <c r="P23" s="39"/>
+      <c r="Q23" s="39"/>
+    </row>
+    <row r="24" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="42">
         <v>46084</v>
       </c>
-      <c r="B21" s="42">
-        <v>1.0416666666666666E-2</v>
-      </c>
-      <c r="C21" s="39">
+      <c r="B24" s="37">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="C24" s="33">
         <f t="shared" si="3"/>
-        <v>0.64583333333333326</v>
-      </c>
-      <c r="D21" s="39">
-        <f t="shared" ref="D21" si="4">C21+B21</f>
-        <v>0.65624999999999989</v>
-      </c>
-      <c r="E21" s="43" t="s">
-        <v>130</v>
-      </c>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="43"/>
-      <c r="I21" s="43"/>
-      <c r="J21" s="43"/>
-      <c r="K21" s="44"/>
-      <c r="L21" s="44"/>
-      <c r="M21" s="44"/>
-      <c r="N21" s="44"/>
-      <c r="O21" s="44"/>
-      <c r="P21" s="44"/>
-    </row>
-    <row r="22" spans="1:16" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="37">
+        <v>0.6875</v>
+      </c>
+      <c r="D24" s="33">
+        <f t="shared" si="0"/>
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="E24" s="38" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="38" t="s">
+        <v>127</v>
+      </c>
+      <c r="G24" s="38" t="s">
+        <v>74</v>
+      </c>
+      <c r="H24" s="38" t="s">
+        <v>74</v>
+      </c>
+      <c r="I24" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J24" s="38" t="s">
+        <v>160</v>
+      </c>
+      <c r="K24" s="38"/>
+      <c r="L24" s="39"/>
+      <c r="M24" s="39"/>
+      <c r="N24" s="39"/>
+      <c r="O24" s="39"/>
+      <c r="P24" s="39"/>
+      <c r="Q24" s="39"/>
+    </row>
+    <row r="25" spans="1:17" ht="115.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="42">
         <v>46084</v>
       </c>
-      <c r="B22" s="42">
+      <c r="B25" s="37">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="C22" s="39">
+      <c r="C25" s="33">
         <f t="shared" si="3"/>
-        <v>0.65624999999999989</v>
-      </c>
-      <c r="D22" s="39">
-        <f t="shared" ref="D22" si="5">C22+B22</f>
-        <v>0.67708333333333326</v>
-      </c>
-      <c r="E22" s="43" t="s">
-        <v>139</v>
-      </c>
-      <c r="F22" s="45"/>
-      <c r="G22" s="43" t="s">
-        <v>132</v>
-      </c>
-      <c r="H22" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I22" s="43"/>
-      <c r="J22" s="43"/>
-      <c r="K22" s="44"/>
-      <c r="L22" s="44"/>
-      <c r="M22" s="44"/>
-      <c r="N22" s="44"/>
-      <c r="O22" s="44"/>
-      <c r="P22" s="44"/>
-    </row>
-    <row r="23" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="37">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D25" s="33">
+        <f t="shared" si="0"/>
+        <v>0.72916666666666674</v>
+      </c>
+      <c r="E25" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="F25" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="G25" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="H25" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="I25" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J25" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="K25" s="38"/>
+      <c r="L25" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="M25" s="39"/>
+      <c r="N25" s="39"/>
+      <c r="O25" s="39"/>
+      <c r="P25" s="39"/>
+      <c r="Q25" s="39"/>
+    </row>
+    <row r="26" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="42">
         <v>46084</v>
       </c>
-      <c r="B23" s="42">
-        <v>3.125E-2</v>
-      </c>
-      <c r="C23" s="39">
+      <c r="B26" s="37">
+        <v>6.25E-2</v>
+      </c>
+      <c r="C26" s="33">
         <f t="shared" si="3"/>
-        <v>0.67708333333333326</v>
-      </c>
-      <c r="D23" s="39">
+        <v>0.72916666666666674</v>
+      </c>
+      <c r="D26" s="33">
         <f t="shared" si="0"/>
-        <v>0.70833333333333326</v>
-      </c>
-      <c r="E23" s="43" t="s">
-        <v>95</v>
-      </c>
-      <c r="F23" s="43" t="s">
-        <v>96</v>
-      </c>
-      <c r="G23" s="43" t="s">
-        <v>132</v>
-      </c>
-      <c r="H23" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I23" s="43"/>
-      <c r="J23" s="43"/>
-      <c r="K23" s="44"/>
-      <c r="L23" s="44"/>
-      <c r="M23" s="44"/>
-      <c r="N23" s="44"/>
-      <c r="O23" s="44"/>
-      <c r="P23" s="44"/>
-    </row>
-    <row r="24" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="37">
+        <v>0.79166666666666674</v>
+      </c>
+      <c r="E26" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="H26" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="I26" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J26" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="K26" s="38"/>
+      <c r="L26" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="M26" s="39"/>
+      <c r="N26" s="39"/>
+      <c r="O26" s="39"/>
+      <c r="P26" s="39"/>
+      <c r="Q26" s="39"/>
+    </row>
+    <row r="27" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="42">
         <v>46084</v>
       </c>
-      <c r="B24" s="42">
-        <v>3.125E-2</v>
-      </c>
-      <c r="C24" s="39">
-        <f t="shared" si="3"/>
-        <v>0.70833333333333326</v>
-      </c>
-      <c r="D24" s="39">
+      <c r="B27" s="37">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="C27" s="33">
+        <f t="shared" si="2"/>
+        <v>0.79166666666666674</v>
+      </c>
+      <c r="D27" s="33">
         <f t="shared" si="0"/>
-        <v>0.73958333333333326</v>
-      </c>
-      <c r="E24" s="43" t="s">
-        <v>97</v>
-      </c>
-      <c r="F24" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="G24" s="43" t="s">
-        <v>132</v>
-      </c>
-      <c r="H24" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I24" s="43"/>
-      <c r="J24" s="43"/>
-      <c r="K24" s="44"/>
-      <c r="L24" s="44"/>
-      <c r="M24" s="44"/>
-      <c r="N24" s="44"/>
-      <c r="O24" s="44"/>
-      <c r="P24" s="44"/>
-    </row>
-    <row r="25" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="37">
-        <v>46084</v>
-      </c>
-      <c r="B25" s="42">
-        <v>3.125E-2</v>
-      </c>
-      <c r="C25" s="39">
-        <f t="shared" si="3"/>
-        <v>0.73958333333333326</v>
-      </c>
-      <c r="D25" s="39">
-        <f t="shared" si="0"/>
-        <v>0.77083333333333326</v>
-      </c>
-      <c r="E25" s="43" t="s">
-        <v>103</v>
-      </c>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43" t="s">
-        <v>118</v>
-      </c>
-      <c r="H25" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I25" s="43"/>
-      <c r="J25" s="43"/>
-      <c r="K25" s="44" t="s">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="E27" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="H27" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="I27" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="J27" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="K27" s="38"/>
+      <c r="L27" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="L25" s="44"/>
-      <c r="M25" s="44"/>
-      <c r="N25" s="44"/>
-      <c r="O25" s="44"/>
-      <c r="P25" s="44"/>
-    </row>
-    <row r="26" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="37">
-        <v>46084</v>
-      </c>
-      <c r="B26" s="42">
-        <v>6.25E-2</v>
-      </c>
-      <c r="C26" s="39">
-        <f t="shared" si="3"/>
-        <v>0.77083333333333326</v>
-      </c>
-      <c r="D26" s="39">
-        <f t="shared" si="0"/>
-        <v>0.83333333333333326</v>
-      </c>
-      <c r="E26" s="43" t="s">
-        <v>115</v>
-      </c>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43" t="s">
-        <v>118</v>
-      </c>
-      <c r="H26" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I26" s="43"/>
-      <c r="J26" s="43"/>
-      <c r="K26" s="44" t="s">
-        <v>53</v>
-      </c>
-      <c r="L26" s="44"/>
-      <c r="M26" s="44"/>
-      <c r="N26" s="44"/>
-      <c r="O26" s="44"/>
-      <c r="P26" s="44"/>
-    </row>
-    <row r="27" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="37">
-        <v>46084</v>
-      </c>
-      <c r="B27" s="42">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C27" s="39">
-        <f t="shared" si="2"/>
-        <v>0.83333333333333326</v>
-      </c>
-      <c r="D27" s="39">
-        <f t="shared" si="0"/>
-        <v>0.87499999999999989</v>
-      </c>
-      <c r="E27" s="43" t="s">
-        <v>108</v>
-      </c>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43" t="s">
-        <v>118</v>
-      </c>
-      <c r="H27" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="I27" s="43"/>
-      <c r="J27" s="43"/>
-      <c r="K27" s="44" t="s">
-        <v>53</v>
-      </c>
-      <c r="L27" s="44"/>
-      <c r="M27" s="44"/>
-      <c r="N27" s="44"/>
-      <c r="O27" s="44"/>
-      <c r="P27" s="44"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B28" s="29"/>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B29" s="29"/>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B30" s="29"/>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B31" s="29"/>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B32" s="29"/>
+      <c r="M27" s="39"/>
+      <c r="N27" s="39"/>
+      <c r="O27" s="39"/>
+      <c r="P27" s="39"/>
+      <c r="Q27" s="39"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="B28" s="44"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="B29" s="44"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="B30" s="44"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="B31" s="44"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="B32" s="44"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B33" s="29"/>
+      <c r="B33" s="44"/>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B34" s="29"/>
+      <c r="B34" s="44"/>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B35" s="31"/>
+      <c r="B35" s="46"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="P28:P162 S4:S20 S21:S62">
+    <dataValidation type="list" allowBlank="1" sqref="Q28:Q162 S4:S62">
       <formula1>"Planned,In Progress,Completed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2247,23 +2458,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="46" t="s">
-        <v>150</v>
-      </c>
-      <c r="B1" s="46" t="s">
-        <v>151</v>
+      <c r="A1" s="48" t="s">
+        <v>171</v>
+      </c>
+      <c r="B1" s="48" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="B2" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
After adding extra places to places to visit in chennai
</commit_message>
<xml_diff>
--- a/config/Agenda.xlsx
+++ b/config/Agenda.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="177">
   <si>
     <t>Client Name</t>
   </si>
@@ -593,6 +593,12 @@
   </si>
   <si>
     <t>Date, Duration(Mins), Start Time, End Time, Session Title, Objective</t>
+  </si>
+  <si>
+    <t>Objective_Visit</t>
+  </si>
+  <si>
+    <t>S.No, Topic, Description</t>
   </si>
 </sst>
 </file>
@@ -719,7 +725,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -855,6 +861,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1246,7 +1253,7 @@
       <c r="B1" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="22" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2450,7 +2457,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.08984375" bestFit="1" customWidth="1"/>
@@ -2466,10 +2473,18 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" s="49" t="s">
+        <v>175</v>
+      </c>
+      <c r="B2" s="49" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>173</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>174</v>
       </c>
     </row>

</xml_diff>

<commit_message>
After going live --- 1. removed login page 2. updated og tags
</commit_message>
<xml_diff>
--- a/config/Agenda.xlsx
+++ b/config/Agenda.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="162">
   <si>
     <t>Client Name</t>
   </si>
@@ -326,18 +326,28 @@
     <t>Changepond Corporate Overiew</t>
   </si>
   <si>
+    <t>Changepond Leadership Update</t>
+  </si>
+  <si>
     <t>Manuel &amp; Ino</t>
   </si>
   <si>
     <t>Changepond Participants</t>
   </si>
   <si>
+    <t>New Initiatives - Demo</t>
+  </si>
+  <si>
+    <t>POC 1 : Dynamic Personalized Offer Engine
+POC 2 : Shop by Emotion
+POC 3 :Real time operational Dashboard view 
+POC 4 : Orders screen - Intelligent priority sorting using color coding 
+POC 5 : QA POC's</t>
+  </si>
+  <si>
     <t>Ideathon 2.0</t>
   </si>
   <si>
-    <t>Sara / Pothy</t>
-  </si>
-  <si>
     <t>Danny</t>
   </si>
   <si>
@@ -356,14 +366,6 @@
     <t xml:space="preserve">Traditional </t>
   </si>
   <si>
-    <t xml:space="preserve">Meet and Greet by Changepond Leadership
-Welcome guest - Meet Leadership Team &amp; Project Team
-</t>
-  </si>
-  <si>
-    <t>Topic 3: PWA - Umbraco - Our Capabilities</t>
-  </si>
-  <si>
     <t xml:space="preserve">Team Dinner </t>
   </si>
   <si>
@@ -388,6 +390,15 @@
     <t xml:space="preserve">Team Building at Turf </t>
   </si>
   <si>
+    <t>Akhilesh, Gopal, Sakthivel</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Leadership Team</t>
+  </si>
+  <si>
     <t>Changepond's experience in offering QA Organizatin setup for other customer - Our Approach, Framework &amp; Methodology, AI in QA Offerings, Governance &amp; Metrics, Risk &amp; Challenges</t>
   </si>
   <si>
@@ -418,10 +429,7 @@
     <t>Coffee Break</t>
   </si>
   <si>
-    <t>Interaction with the team : What went well in 2026 and what are the improvements</t>
-  </si>
-  <si>
-    <t>Godwin &amp; Prasath</t>
+    <t>OMS Team</t>
   </si>
   <si>
     <t>Anil, Selva, SaravanaPandy</t>
@@ -474,113 +482,62 @@
     <t>Duration(Mins)</t>
   </si>
   <si>
-    <t>Coffee Break, Tree Planting. Facility Visit (GCC), Team Photo</t>
-  </si>
-  <si>
-    <t>Changepond Leadership Presentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Topic 4 : CLAP Framework - Agentic Model </t>
-  </si>
-  <si>
-    <t>Topic 5 : Accelerate Knowledge Acquisition Techniques (Use of AI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Akhilesh, Gopal, </t>
-  </si>
-  <si>
-    <t>Gopal</t>
-  </si>
-  <si>
-    <t>Krishna Prasath</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kishore </t>
-  </si>
-  <si>
-    <t>New Initiatives - Demo &amp; Predictive Intelligience Dashboard</t>
-  </si>
-  <si>
-    <t>Pothy /KalaRaj</t>
-  </si>
-  <si>
-    <t>Topic 6: (Placeholder - Topic TBD)</t>
-  </si>
-  <si>
-    <t>Balaji D, Nagaraj , Sara, Katta</t>
-  </si>
-  <si>
-    <t>Anil, Selva, SaravanaPandy , Sara</t>
-  </si>
-  <si>
-    <t>Akhilesh, Gopal, Sara, Selva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Selva or Dhinkar or SP </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sara ,
-( Have to check the Availability of Leadership team) </t>
-  </si>
-  <si>
-    <t>Sara, Selva, Danny, Godwin , KrishnaPrasath , Dhinakar, Amol</t>
-  </si>
-  <si>
-    <t>Sara, Selva,  Godwin , KrishnaPrasath , Prasath</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kalaraj , Pothy, Sara, Selva </t>
-  </si>
-  <si>
-    <t>Amol</t>
-  </si>
-  <si>
-    <t>OMS team , Sara, Selva</t>
-  </si>
-  <si>
-    <t>Sara, Selva, SP,</t>
-  </si>
-  <si>
-    <t>David /Amol</t>
-  </si>
-  <si>
-    <t>Sara, Selva, Amol, Akhilesh ,Dhinakar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prize disttibution to Team 
-Memento to Clients </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entire Team </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Predictive Intelligience Dashboard
-POC 1 : Dynamic Personalized Offer Engine
-POC 2 : Shop by Emotion
-POC 3 :Real time operational Dashboard view 
-POC 4 : Orders screen - Intelligent priority sorting using color coding 
-</t>
-  </si>
-  <si>
-    <t>Selva, SP, Dhinakar</t>
-  </si>
-  <si>
-    <t>Session Presenter</t>
-  </si>
-  <si>
-    <t>Session Owner</t>
-  </si>
-  <si>
-    <t>Kishore</t>
-  </si>
-  <si>
-    <t>Catering Facility</t>
-  </si>
-  <si>
-    <t>Catering Facility , Admin</t>
-  </si>
-  <si>
-    <t>Balaji D, Nagaraj ,  Katta, Anil</t>
+    <t>Nagaraj</t>
+  </si>
+  <si>
+    <t>Balaji D, Nagaraj, Saravana</t>
+  </si>
+  <si>
+    <t>Meet and Greet by Changepond Leadership
+Welcome guest - Meet Leadership Team &amp; Project Team</t>
+  </si>
+  <si>
+    <t>Traditional Lunch</t>
+  </si>
+  <si>
+    <t>Travel to Dakshinachitra</t>
+  </si>
+  <si>
+    <t>Travel from changepond team to Fisherman Cove and then to Dakshinachitra</t>
+  </si>
+  <si>
+    <t>Travel to Mahabalipuram</t>
+  </si>
+  <si>
+    <t>Travel to Manabalipuram</t>
+  </si>
+  <si>
+    <t>Fisherman’s Cove to Changepond</t>
+  </si>
+  <si>
+    <t>Kalaraj, Dhinakar</t>
+  </si>
+  <si>
+    <t>Godwin, Krishnaprasath, Prasath</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLAP Framework - Agentic Model </t>
+  </si>
+  <si>
+    <t>Accelerate Knowledge Acquisition Techniques (Use of AI)</t>
+  </si>
+  <si>
+    <t>PWA - Umbraco - Our Capabilities</t>
+  </si>
+  <si>
+    <t>Tree Planting. Facility Visit (SIX GCC), Team Photo</t>
+  </si>
+  <si>
+    <t>Leadership Meet</t>
+  </si>
+  <si>
+    <t>Meeting Chairman and CEO</t>
+  </si>
+  <si>
+    <t>Interaction with the team : What went well in 2025 and what are the improvements for 2026</t>
+  </si>
+  <si>
+    <t>Receive at Changepond Office</t>
   </si>
   <si>
     <t xml:space="preserve">Sheet name </t>
@@ -593,12 +550,6 @@
   </si>
   <si>
     <t>Date, Duration(Mins), Start Time, End Time, Session Title, Objective</t>
-  </si>
-  <si>
-    <t>Objective_Visit</t>
-  </si>
-  <si>
-    <t>S.No, Topic, Description</t>
   </si>
 </sst>
 </file>
@@ -725,7 +676,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -861,7 +812,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1238,7 +1188,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A2:C6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.1796875" bestFit="1" customWidth="1"/>
@@ -1246,59 +1196,59 @@
     <col min="3" max="3" width="88.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.45">
-      <c r="A1" s="22" t="s">
+    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.45">
+      <c r="A2" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="22" t="s">
-        <v>131</v>
-      </c>
-      <c r="C1" s="22" t="s">
+      <c r="B2" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="23" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="80" x14ac:dyDescent="0.45">
-      <c r="A2" s="23">
+    <row r="3" spans="1:3" ht="80" x14ac:dyDescent="0.45">
+      <c r="A3" s="23">
         <v>1</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B3" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="25" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="80" x14ac:dyDescent="0.35">
-      <c r="A3" s="24">
+      <c r="C3" s="25" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="80" x14ac:dyDescent="0.35">
+      <c r="A4" s="24">
         <v>2</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B4" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="25" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="64" x14ac:dyDescent="0.45">
-      <c r="A4" s="23">
+      <c r="C4" s="25" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="64" x14ac:dyDescent="0.45">
+      <c r="A5" s="23">
         <v>3</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B5" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="26" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="48" x14ac:dyDescent="0.45">
-      <c r="A5" s="23">
+      <c r="C5" s="26" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="48" x14ac:dyDescent="0.45">
+      <c r="A6" s="23">
         <v>4</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B6" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="26" t="s">
-        <v>135</v>
+      <c r="C6" s="26" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1309,7 +1259,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.54296875" style="43" customWidth="1"/>
@@ -1317,24 +1267,24 @@
     <col min="3" max="3" width="11.26953125" style="45" customWidth="1"/>
     <col min="4" max="4" width="11.1796875" style="20" customWidth="1"/>
     <col min="5" max="5" width="42.1796875" style="21" customWidth="1"/>
-    <col min="6" max="6" width="56.7265625" style="21" customWidth="1"/>
-    <col min="7" max="8" width="20.7265625" style="21" customWidth="1"/>
-    <col min="9" max="9" width="17.453125" style="21" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="17.453125" style="21" customWidth="1"/>
-    <col min="12" max="12" width="25.54296875" style="21" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="21" style="21" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="7" style="21" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="10.453125" style="21" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="54.453125" style="21" hidden="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.1796875" style="21"/>
+    <col min="6" max="6" width="64.453125" style="21" customWidth="1"/>
+    <col min="7" max="7" width="27.26953125" style="21" customWidth="1"/>
+    <col min="8" max="8" width="17.453125" style="21" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="17.453125" style="21" customWidth="1"/>
+    <col min="11" max="11" width="25.54296875" style="21" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="21" style="21" hidden="1" customWidth="1"/>
+    <col min="13" max="14" width="7" style="21" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="10.453125" style="21" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="54.453125" style="21" hidden="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.1796875" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="20" customFormat="1" ht="49.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" s="20" customFormat="1" ht="49.5" x14ac:dyDescent="0.35">
       <c r="A1" s="27" t="s">
         <v>5</v>
       </c>
       <c r="B1" s="28" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C1" s="27" t="s">
         <v>88</v>
@@ -1349,40 +1299,37 @@
         <v>10</v>
       </c>
       <c r="G1" s="29" t="s">
-        <v>165</v>
+        <v>11</v>
       </c>
       <c r="H1" s="29" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="I1" s="29" t="s">
-        <v>12</v>
+        <v>94</v>
       </c>
       <c r="J1" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="K1" s="29" t="s">
         <v>90</v>
       </c>
+      <c r="K1" s="30" t="s">
+        <v>13</v>
+      </c>
       <c r="L1" s="30" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M1" s="30" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="N1" s="30" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O1" s="30" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
       <c r="P1" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q1" s="30" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="36" customFormat="1" ht="33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="31">
         <v>46083</v>
       </c>
@@ -1397,23 +1344,20 @@
         <v>87</v>
       </c>
       <c r="F2" s="34" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G2" s="34"/>
       <c r="H2" s="34"/>
-      <c r="I2" s="38" t="s">
-        <v>22</v>
-      </c>
+      <c r="I2" s="34"/>
       <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
+      <c r="K2" s="35"/>
       <c r="L2" s="35"/>
       <c r="M2" s="35"/>
       <c r="N2" s="35"/>
       <c r="O2" s="35"/>
       <c r="P2" s="35"/>
-      <c r="Q2" s="35"/>
-    </row>
-    <row r="3" spans="1:17" s="36" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:16" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="31">
         <v>46083</v>
       </c>
@@ -1432,24 +1376,17 @@
       </c>
       <c r="F3" s="34"/>
       <c r="G3" s="34"/>
-      <c r="H3" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="I3" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J3" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="K3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="35"/>
       <c r="L3" s="35"/>
       <c r="M3" s="35"/>
       <c r="N3" s="35"/>
       <c r="O3" s="35"/>
       <c r="P3" s="35"/>
-      <c r="Q3" s="35"/>
-    </row>
-    <row r="4" spans="1:17" ht="49.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="31">
         <v>46083</v>
       </c>
@@ -1461,40 +1398,37 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="D4" s="33">
-        <f t="shared" ref="D4:D27" si="0">C4+B4</f>
+        <f t="shared" ref="D4:D30" si="0">C4+B4</f>
         <v>0.47916666666666663</v>
       </c>
-      <c r="E4" s="38" t="s">
-        <v>39</v>
+      <c r="E4" s="34" t="s">
+        <v>157</v>
       </c>
       <c r="F4" s="38" t="s">
-        <v>102</v>
-      </c>
-      <c r="G4" s="38"/>
+        <v>141</v>
+      </c>
+      <c r="G4" s="38" t="s">
+        <v>140</v>
+      </c>
       <c r="H4" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="I4" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J4" s="38" t="s">
-        <v>164</v>
-      </c>
-      <c r="K4" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I4" s="38"/>
+      <c r="J4" s="38"/>
+      <c r="K4" s="39" t="s">
+        <v>42</v>
+      </c>
       <c r="L4" s="39" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="M4" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="N4" s="39" t="s">
         <v>41</v>
       </c>
+      <c r="N4" s="39"/>
       <c r="O4" s="39"/>
       <c r="P4" s="39"/>
-      <c r="Q4" s="39"/>
-    </row>
-    <row r="5" spans="1:17" ht="33" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="31">
         <v>46083</v>
       </c>
@@ -1502,7 +1436,7 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="C5" s="33">
-        <f t="shared" ref="C5:C10" si="1">D4</f>
+        <f t="shared" ref="C5:C14" si="1">D4</f>
         <v>0.47916666666666663</v>
       </c>
       <c r="D5" s="33">
@@ -1510,36 +1444,31 @@
         <v>0.49999999999999994</v>
       </c>
       <c r="E5" s="38" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F5" s="40" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H5" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="39" t="s">
+        <v>45</v>
+      </c>
+      <c r="L5" s="39"/>
+      <c r="M5" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="I5" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="K5" s="38"/>
-      <c r="L5" s="39" t="s">
-        <v>45</v>
-      </c>
-      <c r="M5" s="39"/>
-      <c r="N5" s="39" t="s">
-        <v>41</v>
-      </c>
+      <c r="N5" s="39"/>
       <c r="O5" s="39"/>
       <c r="P5" s="39"/>
-      <c r="Q5" s="39"/>
-    </row>
-    <row r="6" spans="1:17" ht="33" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="31">
         <v>46083</v>
       </c>
@@ -1555,36 +1484,31 @@
         <v>0.52083333333333326</v>
       </c>
       <c r="E6" s="38" t="s">
-        <v>138</v>
+        <v>92</v>
       </c>
       <c r="F6" s="40" t="s">
         <v>91</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>40</v>
+        <v>139</v>
       </c>
       <c r="H6" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="I6" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J6" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="K6" s="38"/>
-      <c r="L6" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="38"/>
+      <c r="J6" s="38"/>
+      <c r="K6" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="M6" s="39"/>
-      <c r="N6" s="39" t="s">
+      <c r="L6" s="39"/>
+      <c r="M6" s="39" t="s">
         <v>41</v>
       </c>
+      <c r="N6" s="39"/>
       <c r="O6" s="39"/>
       <c r="P6" s="39"/>
-      <c r="Q6" s="39"/>
-    </row>
-    <row r="7" spans="1:17" ht="33" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="31">
         <v>46083</v>
       </c>
@@ -1603,29 +1527,22 @@
         <v>51</v>
       </c>
       <c r="F7" s="38" t="s">
-        <v>101</v>
-      </c>
-      <c r="G7" s="38" t="s">
-        <v>168</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="G7" s="38"/>
       <c r="H7" s="38" t="s">
-        <v>144</v>
-      </c>
-      <c r="I7" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J7" s="38" t="s">
-        <v>148</v>
-      </c>
-      <c r="K7" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I7" s="38"/>
+      <c r="J7" s="38"/>
+      <c r="K7" s="39"/>
       <c r="L7" s="39"/>
       <c r="M7" s="39"/>
       <c r="N7" s="39"/>
       <c r="O7" s="39"/>
       <c r="P7" s="39"/>
-      <c r="Q7" s="39"/>
-    </row>
-    <row r="8" spans="1:17" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="31">
         <v>46083</v>
       </c>
@@ -1641,32 +1558,27 @@
         <v>0.60416666666666652</v>
       </c>
       <c r="E8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="F8" s="40" t="s">
+        <v>115</v>
+      </c>
+      <c r="G8" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="F8" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="G8" s="38" t="s">
-        <v>124</v>
-      </c>
       <c r="H8" s="38" t="s">
-        <v>74</v>
-      </c>
-      <c r="I8" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J8" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="K8" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I8" s="38"/>
+      <c r="J8" s="38"/>
+      <c r="K8" s="39"/>
       <c r="L8" s="39"/>
       <c r="M8" s="39"/>
       <c r="N8" s="39"/>
       <c r="O8" s="39"/>
       <c r="P8" s="39"/>
-      <c r="Q8" s="39"/>
-    </row>
-    <row r="9" spans="1:17" ht="82.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="31">
         <v>46083</v>
       </c>
@@ -1682,224 +1594,197 @@
         <v>0.62499999999999989</v>
       </c>
       <c r="E9" s="38" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F9" s="38" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G9" s="38" t="s">
-        <v>141</v>
+        <v>112</v>
       </c>
       <c r="H9" s="38" t="s">
-        <v>142</v>
-      </c>
-      <c r="I9" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J9" s="38" t="s">
-        <v>150</v>
-      </c>
-      <c r="K9" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I9" s="38"/>
+      <c r="J9" s="38"/>
+      <c r="K9" s="39"/>
       <c r="L9" s="39"/>
       <c r="M9" s="39"/>
       <c r="N9" s="39"/>
       <c r="O9" s="39"/>
       <c r="P9" s="39"/>
-      <c r="Q9" s="39"/>
-    </row>
-    <row r="10" spans="1:17" ht="66" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="31">
         <v>46083</v>
       </c>
       <c r="B10" s="37">
-        <v>6.25E-2</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="C10" s="33">
         <f t="shared" si="1"/>
         <v>0.62499999999999989</v>
       </c>
       <c r="D10" s="33">
-        <f t="shared" si="0"/>
-        <v>0.68749999999999989</v>
+        <f t="shared" ref="D10" si="2">C10+B10</f>
+        <v>0.64583333333333326</v>
       </c>
       <c r="E10" s="41" t="s">
-        <v>115</v>
+        <v>143</v>
       </c>
       <c r="F10" s="40" t="s">
-        <v>116</v>
+        <v>144</v>
       </c>
       <c r="G10" s="38"/>
       <c r="H10" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="I10" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J10" s="38" t="s">
-        <v>151</v>
-      </c>
-      <c r="K10" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I10" s="38"/>
+      <c r="J10" s="38"/>
+      <c r="K10" s="39"/>
       <c r="L10" s="39"/>
       <c r="M10" s="39"/>
       <c r="N10" s="39"/>
       <c r="O10" s="39"/>
       <c r="P10" s="39"/>
-      <c r="Q10" s="39"/>
-    </row>
-    <row r="11" spans="1:17" ht="82.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="31">
         <v>46083</v>
       </c>
       <c r="B11" s="37">
-        <v>0.10416666666666667</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="C11" s="33">
-        <f>D10</f>
-        <v>0.68749999999999989</v>
+        <f t="shared" si="1"/>
+        <v>0.64583333333333326</v>
       </c>
       <c r="D11" s="33">
         <f t="shared" si="0"/>
-        <v>0.79166666666666652</v>
+        <v>0.68749999999999989</v>
       </c>
       <c r="E11" s="41" t="s">
-        <v>23</v>
+        <v>118</v>
       </c>
       <c r="F11" s="40" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G11" s="38"/>
       <c r="H11" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="I11" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J11" s="38" t="s">
-        <v>151</v>
-      </c>
-      <c r="K11" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I11" s="38"/>
+      <c r="J11" s="38"/>
+      <c r="K11" s="39"/>
       <c r="L11" s="39"/>
       <c r="M11" s="39"/>
       <c r="N11" s="39"/>
       <c r="O11" s="39"/>
       <c r="P11" s="39"/>
-      <c r="Q11" s="39"/>
-    </row>
-    <row r="12" spans="1:17" ht="66" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="31">
         <v>46083</v>
       </c>
       <c r="B12" s="37">
-        <v>4.1666666666666664E-2</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="C12" s="33">
-        <f>D11</f>
-        <v>0.79166666666666652</v>
+        <f t="shared" si="1"/>
+        <v>0.68749999999999989</v>
       </c>
       <c r="D12" s="33">
         <f t="shared" si="0"/>
-        <v>0.83333333333333315</v>
-      </c>
-      <c r="E12" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="F12" s="38" t="s">
-        <v>129</v>
+        <v>0.70833333333333326</v>
+      </c>
+      <c r="E12" s="41" t="s">
+        <v>145</v>
+      </c>
+      <c r="F12" s="40" t="s">
+        <v>146</v>
       </c>
       <c r="G12" s="38"/>
       <c r="H12" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="I12" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J12" s="38" t="s">
-        <v>152</v>
-      </c>
-      <c r="K12" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I12" s="38"/>
+      <c r="J12" s="38"/>
+      <c r="K12" s="39"/>
       <c r="L12" s="39"/>
       <c r="M12" s="39"/>
       <c r="N12" s="39"/>
       <c r="O12" s="39"/>
       <c r="P12" s="39"/>
-      <c r="Q12" s="39"/>
-    </row>
-    <row r="13" spans="1:17" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="42">
-        <v>46084</v>
+    </row>
+    <row r="13" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="31">
+        <v>46083</v>
       </c>
       <c r="B13" s="37">
-        <v>2.0833333333333332E-2</v>
+        <v>0.10416666666666667</v>
       </c>
       <c r="C13" s="33">
-        <v>0.39583333333333331</v>
+        <f t="shared" si="1"/>
+        <v>0.70833333333333326</v>
       </c>
       <c r="D13" s="33">
         <f t="shared" si="0"/>
-        <v>0.41666666666666663</v>
-      </c>
-      <c r="E13" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="F13" s="40"/>
+        <v>0.81249999999999989</v>
+      </c>
+      <c r="E13" s="41" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="40" t="s">
+        <v>120</v>
+      </c>
       <c r="G13" s="38"/>
-      <c r="H13" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="I13" s="38" t="s">
-        <v>22</v>
-      </c>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
       <c r="J13" s="38"/>
-      <c r="K13" s="38"/>
+      <c r="K13" s="39"/>
       <c r="L13" s="39"/>
       <c r="M13" s="39"/>
       <c r="N13" s="39"/>
       <c r="O13" s="39"/>
       <c r="P13" s="39"/>
-      <c r="Q13" s="39"/>
-    </row>
-    <row r="14" spans="1:17" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="42">
-        <v>46084</v>
+    </row>
+    <row r="14" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="31">
+        <v>46083</v>
       </c>
       <c r="B14" s="37">
-        <v>3.125E-2</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="C14" s="33">
-        <f>D13</f>
-        <v>0.41666666666666663</v>
+        <f t="shared" si="1"/>
+        <v>0.81249999999999989</v>
       </c>
       <c r="D14" s="33">
         <f t="shared" si="0"/>
-        <v>0.44791666666666663</v>
+        <v>0.89583333333333326</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>103</v>
+        <v>132</v>
       </c>
       <c r="F14" s="38" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="H14" s="38" t="s">
-        <v>96</v>
-      </c>
-      <c r="I14" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J14" s="38" t="s">
-        <v>153</v>
-      </c>
-      <c r="K14" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I14" s="38"/>
+      <c r="J14" s="38"/>
+      <c r="K14" s="39"/>
       <c r="L14" s="39"/>
       <c r="M14" s="39"/>
       <c r="N14" s="39"/>
       <c r="O14" s="39"/>
       <c r="P14" s="39"/>
-      <c r="Q14" s="39"/>
-    </row>
-    <row r="15" spans="1:17" ht="66" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="42">
         <v>46084</v>
       </c>
@@ -1907,40 +1792,32 @@
         <v>3.125E-2</v>
       </c>
       <c r="C15" s="33">
-        <f t="shared" ref="C15:C27" si="2">D14</f>
-        <v>0.44791666666666663</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="D15" s="33">
         <f t="shared" si="0"/>
-        <v>0.47916666666666663</v>
-      </c>
-      <c r="E15" s="38" t="s">
-        <v>139</v>
-      </c>
-      <c r="F15" s="38" t="s">
-        <v>120</v>
-      </c>
-      <c r="G15" s="38" t="s">
-        <v>123</v>
-      </c>
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="G15" s="38"/>
       <c r="H15" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="I15" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J15" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="K15" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I15" s="38"/>
+      <c r="J15" s="38"/>
+      <c r="K15" s="39"/>
       <c r="L15" s="39"/>
       <c r="M15" s="39"/>
       <c r="N15" s="39"/>
       <c r="O15" s="39"/>
       <c r="P15" s="39"/>
-      <c r="Q15" s="39"/>
-    </row>
-    <row r="16" spans="1:17" ht="33" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="42">
         <v>46084</v>
       </c>
@@ -1948,272 +1825,231 @@
         <v>3.125E-2</v>
       </c>
       <c r="C16" s="33">
-        <f t="shared" si="2"/>
-        <v>0.47916666666666663</v>
+        <f>D15</f>
+        <v>0.42708333333333331</v>
       </c>
       <c r="D16" s="33">
-        <f t="shared" si="0"/>
-        <v>0.51041666666666663</v>
+        <f t="shared" ref="D16:D22" si="3">C16+B16</f>
+        <v>0.45833333333333331</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>137</v>
-      </c>
-      <c r="F16" s="38"/>
+        <v>150</v>
+      </c>
+      <c r="F16" s="38" t="s">
+        <v>123</v>
+      </c>
       <c r="G16" s="38" t="s">
-        <v>169</v>
+        <v>149</v>
       </c>
       <c r="H16" s="38" t="s">
-        <v>144</v>
-      </c>
-      <c r="I16" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J16" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="K16" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I16" s="38"/>
+      <c r="J16" s="38"/>
+      <c r="K16" s="39"/>
       <c r="L16" s="39"/>
       <c r="M16" s="39"/>
       <c r="N16" s="39"/>
       <c r="O16" s="39"/>
       <c r="P16" s="39"/>
-      <c r="Q16" s="39"/>
-    </row>
-    <row r="17" spans="1:17" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="42">
         <v>46084</v>
       </c>
       <c r="B17" s="37">
-        <v>3.125E-2</v>
+        <v>1.0416666666666666E-2</v>
       </c>
       <c r="C17" s="33">
-        <f t="shared" si="2"/>
-        <v>0.51041666666666663</v>
+        <f t="shared" ref="C17:C30" si="4">D16</f>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D17" s="33">
-        <f t="shared" si="0"/>
-        <v>0.54166666666666663</v>
+        <f t="shared" si="3"/>
+        <v>0.46875</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="F17" s="38" t="s">
-        <v>119</v>
-      </c>
-      <c r="G17" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="H17" s="38" t="s">
-        <v>146</v>
-      </c>
-      <c r="I17" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J17" s="38" t="s">
-        <v>155</v>
-      </c>
-      <c r="K17" s="38"/>
+        <v>124</v>
+      </c>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="38"/>
+      <c r="J17" s="38"/>
+      <c r="K17" s="39"/>
       <c r="L17" s="39"/>
       <c r="M17" s="39"/>
       <c r="N17" s="39"/>
       <c r="O17" s="39"/>
       <c r="P17" s="39"/>
-      <c r="Q17" s="39"/>
-    </row>
-    <row r="18" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="42">
         <v>46084</v>
       </c>
       <c r="B18" s="37">
-        <v>4.1666666666666664E-2</v>
+        <v>3.125E-2</v>
       </c>
       <c r="C18" s="33">
-        <f t="shared" ref="C18:C26" si="3">D17</f>
-        <v>0.54166666666666663</v>
+        <f t="shared" si="4"/>
+        <v>0.46875</v>
       </c>
       <c r="D18" s="33">
-        <f t="shared" si="0"/>
-        <v>0.58333333333333326</v>
+        <f t="shared" si="3"/>
+        <v>0.5</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>51</v>
+        <v>151</v>
       </c>
       <c r="F18" s="38" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="G18" s="38" t="s">
-        <v>168</v>
+        <v>148</v>
       </c>
       <c r="H18" s="38" t="s">
-        <v>144</v>
-      </c>
-      <c r="I18" s="38" t="s">
-        <v>22</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="I18" s="38"/>
       <c r="J18" s="38"/>
-      <c r="K18" s="38"/>
+      <c r="K18" s="39"/>
       <c r="L18" s="39"/>
       <c r="M18" s="39"/>
       <c r="N18" s="39"/>
       <c r="O18" s="39"/>
       <c r="P18" s="39"/>
-      <c r="Q18" s="39"/>
-    </row>
-    <row r="19" spans="1:17" ht="16.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="42">
         <v>46084</v>
       </c>
       <c r="B19" s="37">
-        <v>2.0833333333333332E-2</v>
+        <v>3.125E-2</v>
       </c>
       <c r="C19" s="33">
+        <f t="shared" si="4"/>
+        <v>0.5</v>
+      </c>
+      <c r="D19" s="33">
         <f t="shared" si="3"/>
-        <v>0.58333333333333326</v>
-      </c>
-      <c r="D19" s="33">
-        <f>C19+B19</f>
-        <v>0.60416666666666663</v>
+        <v>0.53125</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>147</v>
-      </c>
-      <c r="F19" s="40"/>
-      <c r="G19" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="H19" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="I19" s="38" t="s">
-        <v>22</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="F19" s="38"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="38"/>
+      <c r="I19" s="38"/>
       <c r="J19" s="38"/>
-      <c r="K19" s="38"/>
+      <c r="K19" s="39"/>
       <c r="L19" s="39"/>
       <c r="M19" s="39"/>
       <c r="N19" s="39"/>
       <c r="O19" s="39"/>
       <c r="P19" s="39"/>
-      <c r="Q19" s="39"/>
-    </row>
-    <row r="20" spans="1:17" ht="33" x14ac:dyDescent="0.35">
+    </row>
+    <row r="20" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="42">
         <v>46084</v>
       </c>
       <c r="B20" s="37">
-        <v>2.0833333333333332E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="C20" s="33">
+        <f t="shared" si="4"/>
+        <v>0.53125</v>
+      </c>
+      <c r="D20" s="33">
         <f t="shared" si="3"/>
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="D20" s="33">
-        <f t="shared" si="0"/>
-        <v>0.625</v>
+        <v>0.57291666666666663</v>
       </c>
       <c r="E20" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="F20" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="G20" s="38" t="s">
-        <v>156</v>
-      </c>
-      <c r="H20" s="38" t="s">
-        <v>72</v>
-      </c>
-      <c r="I20" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J20" s="38" t="s">
-        <v>157</v>
-      </c>
-      <c r="K20" s="38"/>
+        <v>51</v>
+      </c>
+      <c r="F20" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="G20" s="38"/>
+      <c r="H20" s="38"/>
+      <c r="I20" s="38"/>
+      <c r="J20" s="38"/>
+      <c r="K20" s="39"/>
       <c r="L20" s="39"/>
       <c r="M20" s="39"/>
       <c r="N20" s="39"/>
       <c r="O20" s="39"/>
       <c r="P20" s="39"/>
-      <c r="Q20" s="39"/>
-    </row>
-    <row r="21" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="42">
         <v>46084</v>
       </c>
       <c r="B21" s="37">
-        <v>1.0416666666666666E-2</v>
+        <v>3.125E-2</v>
       </c>
       <c r="C21" s="33">
+        <f t="shared" si="4"/>
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="D21" s="33">
         <f t="shared" si="3"/>
-        <v>0.625</v>
-      </c>
-      <c r="D21" s="33">
-        <f t="shared" ref="D21" si="4">C21+B21</f>
-        <v>0.63541666666666663</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="E21" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="F21" s="38"/>
-      <c r="G21" s="38" t="s">
-        <v>168</v>
-      </c>
-      <c r="H21" s="38" t="s">
-        <v>144</v>
-      </c>
-      <c r="I21" s="38" t="s">
-        <v>22</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="F21" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="G21" s="38"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="38"/>
       <c r="J21" s="38"/>
-      <c r="K21" s="38"/>
+      <c r="K21" s="39"/>
       <c r="L21" s="39"/>
       <c r="M21" s="39"/>
       <c r="N21" s="39"/>
       <c r="O21" s="39"/>
       <c r="P21" s="39"/>
-      <c r="Q21" s="39"/>
-    </row>
-    <row r="22" spans="1:17" ht="16.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="22" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="42">
         <v>46084</v>
       </c>
       <c r="B22" s="37">
-        <v>2.0833333333333332E-2</v>
+        <v>3.125E-2</v>
       </c>
       <c r="C22" s="33">
+        <f t="shared" si="4"/>
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D22" s="33">
         <f t="shared" si="3"/>
         <v>0.63541666666666663</v>
       </c>
-      <c r="D22" s="33">
-        <f t="shared" ref="D22" si="5">C22+B22</f>
-        <v>0.65625</v>
-      </c>
       <c r="E22" s="38" t="s">
-        <v>128</v>
-      </c>
-      <c r="F22" s="40"/>
+        <v>152</v>
+      </c>
+      <c r="F22" s="38" t="s">
+        <v>121</v>
+      </c>
       <c r="G22" s="38" t="s">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="H22" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="I22" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J22" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="K22" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I22" s="38"/>
+      <c r="J22" s="38"/>
+      <c r="K22" s="39"/>
       <c r="L22" s="39"/>
       <c r="M22" s="39"/>
       <c r="N22" s="39"/>
       <c r="O22" s="39"/>
       <c r="P22" s="39"/>
-      <c r="Q22" s="39"/>
-    </row>
-    <row r="23" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="23" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="42">
         <v>46084</v>
       </c>
@@ -2221,81 +2057,65 @@
         <v>3.125E-2</v>
       </c>
       <c r="C23" s="33">
-        <f t="shared" si="3"/>
-        <v>0.65625</v>
+        <f t="shared" si="4"/>
+        <v>0.63541666666666663</v>
       </c>
       <c r="D23" s="33">
         <f t="shared" si="0"/>
-        <v>0.6875</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>145</v>
-      </c>
-      <c r="F23" s="38" t="s">
-        <v>163</v>
+        <v>127</v>
+      </c>
+      <c r="F23" s="40" t="s">
+        <v>156</v>
       </c>
       <c r="G23" s="38" t="s">
-        <v>159</v>
+        <v>125</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>72</v>
-      </c>
-      <c r="I23" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J23" s="38" t="s">
-        <v>157</v>
-      </c>
-      <c r="K23" s="38"/>
+        <v>22</v>
+      </c>
+      <c r="I23" s="38"/>
+      <c r="J23" s="38"/>
+      <c r="K23" s="39"/>
       <c r="L23" s="39"/>
       <c r="M23" s="39"/>
       <c r="N23" s="39"/>
       <c r="O23" s="39"/>
       <c r="P23" s="39"/>
-      <c r="Q23" s="39"/>
-    </row>
-    <row r="24" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="24" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="42">
         <v>46084</v>
       </c>
       <c r="B24" s="37">
-        <v>2.0833333333333332E-2</v>
+        <v>1.0416666666666666E-2</v>
       </c>
       <c r="C24" s="33">
-        <f t="shared" si="3"/>
-        <v>0.6875</v>
+        <f t="shared" si="4"/>
+        <v>0.66666666666666663</v>
       </c>
       <c r="D24" s="33">
-        <f t="shared" si="0"/>
-        <v>0.70833333333333337</v>
+        <f t="shared" ref="D24" si="5">C24+B24</f>
+        <v>0.67708333333333326</v>
       </c>
       <c r="E24" s="38" t="s">
-        <v>94</v>
-      </c>
-      <c r="F24" s="38" t="s">
-        <v>127</v>
-      </c>
-      <c r="G24" s="38" t="s">
-        <v>74</v>
-      </c>
-      <c r="H24" s="38" t="s">
-        <v>74</v>
-      </c>
-      <c r="I24" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J24" s="38" t="s">
-        <v>160</v>
-      </c>
-      <c r="K24" s="38"/>
+        <v>124</v>
+      </c>
+      <c r="F24" s="38"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="38"/>
+      <c r="I24" s="38"/>
+      <c r="J24" s="38"/>
+      <c r="K24" s="39"/>
       <c r="L24" s="39"/>
       <c r="M24" s="39"/>
       <c r="N24" s="39"/>
       <c r="O24" s="39"/>
       <c r="P24" s="39"/>
-      <c r="Q24" s="39"/>
-    </row>
-    <row r="25" spans="1:17" ht="115.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="42">
         <v>46084</v>
       </c>
@@ -2303,136 +2123,216 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="C25" s="33">
-        <f t="shared" si="3"/>
-        <v>0.70833333333333337</v>
+        <f t="shared" si="4"/>
+        <v>0.67708333333333326</v>
       </c>
       <c r="D25" s="33">
-        <f t="shared" si="0"/>
-        <v>0.72916666666666674</v>
+        <f t="shared" ref="D25" si="6">C25+B25</f>
+        <v>0.69791666666666663</v>
       </c>
       <c r="E25" s="38" t="s">
-        <v>99</v>
-      </c>
-      <c r="F25" s="38" t="s">
-        <v>161</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="F25" s="40"/>
       <c r="G25" s="38" t="s">
-        <v>40</v>
+        <v>125</v>
       </c>
       <c r="H25" s="38" t="s">
-        <v>144</v>
-      </c>
-      <c r="I25" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J25" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="K25" s="38"/>
-      <c r="L25" s="39" t="s">
-        <v>53</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="I25" s="38"/>
+      <c r="J25" s="38"/>
+      <c r="K25" s="39"/>
+      <c r="L25" s="39"/>
       <c r="M25" s="39"/>
       <c r="N25" s="39"/>
       <c r="O25" s="39"/>
       <c r="P25" s="39"/>
-      <c r="Q25" s="39"/>
-    </row>
-    <row r="26" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="42">
         <v>46084</v>
       </c>
       <c r="B26" s="37">
-        <v>6.25E-2</v>
+        <v>3.125E-2</v>
       </c>
       <c r="C26" s="33">
-        <f t="shared" si="3"/>
-        <v>0.72916666666666674</v>
+        <f t="shared" si="4"/>
+        <v>0.69791666666666663</v>
       </c>
       <c r="D26" s="33">
         <f t="shared" si="0"/>
-        <v>0.79166666666666674</v>
+        <v>0.72916666666666663</v>
       </c>
       <c r="E26" s="38" t="s">
-        <v>111</v>
-      </c>
-      <c r="F26" s="38"/>
+        <v>95</v>
+      </c>
+      <c r="F26" s="38" t="s">
+        <v>96</v>
+      </c>
       <c r="G26" s="38" t="s">
-        <v>167</v>
+        <v>125</v>
       </c>
       <c r="H26" s="38" t="s">
-        <v>144</v>
-      </c>
-      <c r="I26" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J26" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="K26" s="38"/>
-      <c r="L26" s="39" t="s">
-        <v>53</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="I26" s="38"/>
+      <c r="J26" s="38"/>
+      <c r="K26" s="39"/>
+      <c r="L26" s="39"/>
       <c r="M26" s="39"/>
       <c r="N26" s="39"/>
       <c r="O26" s="39"/>
       <c r="P26" s="39"/>
-      <c r="Q26" s="39"/>
-    </row>
-    <row r="27" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="42">
         <v>46084</v>
       </c>
       <c r="B27" s="37">
-        <v>4.1666666666666664E-2</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="C27" s="33">
-        <f t="shared" si="2"/>
-        <v>0.79166666666666674</v>
+        <f t="shared" si="4"/>
+        <v>0.72916666666666663</v>
       </c>
       <c r="D27" s="33">
         <f t="shared" si="0"/>
-        <v>0.83333333333333337</v>
+        <v>0.75</v>
       </c>
       <c r="E27" s="38" t="s">
-        <v>104</v>
-      </c>
-      <c r="F27" s="38"/>
+        <v>97</v>
+      </c>
+      <c r="F27" s="38" t="s">
+        <v>129</v>
+      </c>
       <c r="G27" s="38" t="s">
-        <v>167</v>
+        <v>125</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>144</v>
-      </c>
-      <c r="I27" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="J27" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="K27" s="38"/>
-      <c r="L27" s="39" t="s">
-        <v>53</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="I27" s="38"/>
+      <c r="J27" s="38"/>
+      <c r="K27" s="39"/>
+      <c r="L27" s="39"/>
       <c r="M27" s="39"/>
       <c r="N27" s="39"/>
       <c r="O27" s="39"/>
       <c r="P27" s="39"/>
-      <c r="Q27" s="39"/>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="B28" s="44"/>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="B29" s="44"/>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="B30" s="44"/>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="28" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="42">
+        <v>46084</v>
+      </c>
+      <c r="B28" s="37">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="C28" s="33">
+        <f t="shared" si="4"/>
+        <v>0.75</v>
+      </c>
+      <c r="D28" s="33">
+        <f t="shared" si="0"/>
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="E28" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="H28" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="I28" s="38"/>
+      <c r="J28" s="38"/>
+      <c r="K28" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="L28" s="39"/>
+      <c r="M28" s="39"/>
+      <c r="N28" s="39"/>
+      <c r="O28" s="39"/>
+      <c r="P28" s="39"/>
+    </row>
+    <row r="29" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="42">
+        <v>46084</v>
+      </c>
+      <c r="B29" s="37">
+        <v>6.25E-2</v>
+      </c>
+      <c r="C29" s="33">
+        <f t="shared" si="4"/>
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="D29" s="33">
+        <f t="shared" si="0"/>
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="E29" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="F29" s="38"/>
+      <c r="G29" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="H29" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="38"/>
+      <c r="J29" s="38"/>
+      <c r="K29" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="L29" s="39"/>
+      <c r="M29" s="39"/>
+      <c r="N29" s="39"/>
+      <c r="O29" s="39"/>
+      <c r="P29" s="39"/>
+    </row>
+    <row r="30" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="42">
+        <v>46084</v>
+      </c>
+      <c r="B30" s="37">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="C30" s="33">
+        <f t="shared" si="4"/>
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="D30" s="33">
+        <f t="shared" si="0"/>
+        <v>0.875</v>
+      </c>
+      <c r="E30" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="H30" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="38"/>
+      <c r="J30" s="38"/>
+      <c r="K30" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="L30" s="39"/>
+      <c r="M30" s="39"/>
+      <c r="N30" s="39"/>
+      <c r="O30" s="39"/>
+      <c r="P30" s="39"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B31" s="44"/>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B32" s="44"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.35">
@@ -2442,11 +2342,20 @@
       <c r="B34" s="44"/>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B35" s="46"/>
+      <c r="B35" s="44"/>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B36" s="44"/>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B37" s="44"/>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B38" s="46"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="Q28:Q162 S4:S62">
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" sqref="P31:P165 S4:S65">
       <formula1>"Planned,In Progress,Completed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2457,7 +2366,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.08984375" bestFit="1" customWidth="1"/>
@@ -2466,26 +2375,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="48" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="B1" s="48" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="49" t="s">
-        <v>175</v>
-      </c>
-      <c r="B2" s="49" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>173</v>
-      </c>
-      <c r="B3" t="s">
-        <v>174</v>
+      <c r="A2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B2" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>